<commit_message>
feat(F-NAR-019): TREE-COL-026 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-COL-026.xlsx
+++ b/stories/arbres/TREE-COL-026.xlsx
@@ -854,7 +854,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Un cerf-volant rouge s'accroche au figuier. Aniss veut le copier sur l'ardoise verte avant le vent. Sa première phrase se perd, la craie casse, sa main se couvre de poussière. Sur le tapis, la table ou la fenêtre, il apprend à attendre la fin des voix. L'éponge, la craie ou le tabouret changent le dessin. Le clou, le pain ou le volet lui donnent enfin des oreilles. Le soir, l'ardoise garde le cerf-volant, et sa main n'est plus trop pressée.</t>
+          <t>Un cerf-volant rouge s'accroche au figuier. Aniss veut le copier sur l'ardoise verte avant le vent. Sa première phrase se perd, la craie casse, sa main se couvre de poussière. Sur le tapis, la table ou la fenêtre, il attend la fin des voix. L'éponge, la craie ou le tabouret changent le dessin. Le clou, le pain ou le volet lui donnent enfin des oreilles. Le soir, l'ardoise garde le cerf-volant, et sa main n'est plus trop pressée.</t>
         </is>
       </c>
     </row>
@@ -2933,17 +2933,17 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec l'éponge, puis le clou. On a entendu toute ta phrase. Sa paume est propre, un peu froide. Une goutte tombe du clou, sur la laine grise.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec l'éponge, puis le clou. Tes mots sont arrivés, cette fois. Sa paume est propre, un peu froide. Une goutte tombe du clou, sur la laine grise.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec l'éponge, puis le clou. On a entendu toute ta phrase. Sa paume est propre, un peu froide. Une goutte tombe du clou, sur la laine grise.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec l'éponge, puis le clou. Tes mots sont arrivés, cette fois. Sa paume est propre, un peu froide. Une goutte tombe du clou, sur la laine grise.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec l'éponge, puis le clou. On a entendu toute ta phrase. Sa paume est propre, un peu froide. Une goutte tombe du clou, sur la laine grise.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec l'éponge, puis le clou. Tes mots sont arrivés, cette fois. Sa paume est propre, un peu froide. Une goutte tombe du clou, sur la laine grise.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -3081,7 +3081,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné sur le tapis, avec l'éponge, puis le clou.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Sa paume est propre, un peu froide.
 narrateur|Une goutte tombe du clou, sur la laine grise.</t>
         </is>
@@ -3303,17 +3303,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec l'éponge, puis le pain. On a entendu toute ta phrase. Sa paume est propre, un peu froide. L'éponge humide garde une miette de pain.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec l'éponge, puis le pain. Tes mots sont arrivés, cette fois. Sa paume est propre, un peu froide. L'éponge humide garde une miette de pain.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec l'éponge, puis le pain. On a entendu toute ta phrase. Sa paume est propre, un peu froide. L'éponge humide garde une miette de pain.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec l'éponge, puis le pain. Tes mots sont arrivés, cette fois. Sa paume est propre, un peu froide. L'éponge humide garde une miette de pain.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec l'éponge, puis le pain. On a entendu toute ta phrase. Sa paume est propre, un peu froide. L'éponge humide garde une miette de pain.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec l'éponge, puis le pain. Tes mots sont arrivés, cette fois. Sa paume est propre, un peu froide. L'éponge humide garde une miette de pain.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -3451,7 +3451,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné sur le tapis, avec l'éponge, puis le pain.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Sa paume est propre, un peu froide.
 narrateur|L'éponge humide garde une miette de pain.</t>
         </is>
@@ -3673,17 +3673,17 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec l'éponge, puis le volet. On a entendu toute ta phrase. Sa paume est propre, un peu froide. Sur le tapis, l'éponge sèche près du volet ouvert.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec l'éponge, puis le volet. Tes mots sont arrivés, cette fois. Sa paume est propre, un peu froide. Sur le tapis, l'éponge sèche près du volet ouvert.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec l'éponge, puis le volet. On a entendu toute ta phrase. Sa paume est propre, un peu froide. Sur le tapis, l'éponge sèche près du volet ouvert.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec l'éponge, puis le volet. Tes mots sont arrivés, cette fois. Sa paume est propre, un peu froide. Sur le tapis, l'éponge sèche près du volet ouvert.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec l'éponge, puis le volet. On a entendu toute ta phrase. Sa paume est propre, un peu froide. Sur le tapis, l'éponge sèche près du volet ouvert.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec l'éponge, puis le volet. Tes mots sont arrivés, cette fois. Sa paume est propre, un peu froide. Sur le tapis, l'éponge sèche près du volet ouvert.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr"/>
@@ -3821,7 +3821,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné sur le tapis, avec l'éponge, puis le volet.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Sa paume est propre, un peu froide.
 narrateur|Sur le tapis, l'éponge sèche près du volet ouvert.</t>
         </is>
@@ -4433,17 +4433,17 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec la craie neuve, puis le clou. On a entendu toute ta phrase. Un croissant jaune reste au creux de sa main. Un grain de craie jaune dort sous le clou.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec la craie neuve, puis le clou. Tes mots sont arrivés, cette fois. Un croissant jaune reste au creux de sa main. Un grain de craie jaune dort sous le clou.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec la craie neuve, puis le clou. On a entendu toute ta phrase. Un croissant jaune reste au creux de sa main. Un grain de craie jaune dort sous le clou.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec la craie neuve, puis le clou. Tes mots sont arrivés, cette fois. Un croissant jaune reste au creux de sa main. Un grain de craie jaune dort sous le clou.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec la craie neuve, puis le clou. On a entendu toute ta phrase. Un croissant jaune reste au creux de sa main. Un grain de craie jaune dort sous le clou.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec la craie neuve, puis le clou. Tes mots sont arrivés, cette fois. Un croissant jaune reste au creux de sa main. Un grain de craie jaune dort sous le clou.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
@@ -4581,7 +4581,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné sur le tapis, avec la craie neuve, puis le clou.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Un croissant jaune reste au creux de sa main.
 narrateur|Un grain de craie jaune dort sous le clou.</t>
         </is>
@@ -4615,17 +4615,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Aniss pose l'ardoise à côté de la croûte. La craie jaune roule vers le pain. Attention, ma ligne ! Maman rit d'une phrase de papa. Personne n'a vu la craie. Aniss la rattrape, puis il attend. Pardon, on était loin. Montre ton trait. Le jaune, c'est le soleil sur le rouge. On croirait le figuier, en miniature. Farine et craie se touchent, sur sa main. Deux blancs différents, l'un chaud, l'un sec. Le pain peut veiller le dessin.</t>
+          <t>Aniss pose l'ardoise à côté de la croûte. La craie jaune roule vers le pain. Attention, ma ligne ! Maman rit d'une phrase de papa. Personne n'a vu la craie. Aniss la rattrape, puis il attend. Pardon, on était loin. Montre ton trait. Le jaune, c'est le soleil sur le rouge. On dirait le figuier, plus petit. Farine et craie se touchent, sur sa main. Deux blancs différents, l'un chaud, l'un sec. Le pain peut veiller le dessin.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss pose l'ardoise à côté de la croûte. La craie jaune roule vers le pain. Attention, ma ligne ! Maman rit d'une phrase de papa. Personne n'a vu la craie. Aniss la rattrape, puis il attend. Pardon, on était loin. Montre ton trait. Le jaune, c'est le soleil sur le rouge. On croirait le figuier, en miniature. Farine et craie se touchent, sur sa main. Deux blancs différents, l'un chaud, l'un sec. Le pain peut veiller le dessin.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss pose l'ardoise à côté de la croûte. La craie jaune roule vers le pain. Attention, ma ligne ! Maman rit d'une phrase de papa. Personne n'a vu la craie. Aniss la rattrape, puis il attend. Pardon, on était loin. Montre ton trait. Le jaune, c'est le soleil sur le rouge. On dirait le figuier, plus petit. Farine et craie se touchent, sur sa main. Deux blancs différents, l'un chaud, l'un sec. Le pain peut veiller le dessin.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Aniss pose l'ardoise à côté de la croûte. La craie jaune roule vers le pain. Attention, ma ligne ! Maman rit d'une phrase de papa. Personne n'a vu la craie. Aniss la rattrape, puis il attend. Pardon, on était loin. Montre ton trait. Le jaune, c'est le soleil sur le rouge. On croirait le figuier, en miniature. Farine et craie se touchent, sur sa main. Deux blancs différents, l'un chaud, l'un sec. Le pain peut veiller le dessin. [pause]</t>
+          <t>Aniss pose l'ardoise à côté de la croûte. La craie jaune roule vers le pain. Attention, ma ligne ! Maman rit d'une phrase de papa. Personne n'a vu la craie. Aniss la rattrape, puis il attend. Pardon, on était loin. Montre ton trait. Le jaune, c'est le soleil sur le rouge. On dirait le figuier, plus petit. Farine et craie se touchent, sur sa main. Deux blancs différents, l'un chaud, l'un sec. Le pain peut veiller le dessin. [pause]</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -4768,7 +4768,7 @@
 maman|Pardon, on était loin.
 maman|Montre ton trait.
 enfant-m|Le jaune, c'est le soleil sur le rouge.
-papa|On croirait le figuier, en miniature.
+papa|On dirait le figuier, plus petit.
 narrateur|Farine et craie se touchent, sur sa main.
 narrateur|Deux blancs différents, l'un chaud, l'un sec.
 maman|Le pain peut veiller le dessin.</t>
@@ -4803,17 +4803,17 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec la craie neuve, puis le pain. On a entendu toute ta phrase. Un croissant jaune reste au creux de sa main. La croûte et la craie sentent le chaud, toutes les deux.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec la craie neuve, puis le pain. Tes mots sont arrivés, cette fois. Un croissant jaune reste au creux de sa main. La croûte et la craie sentent le chaud, toutes les deux.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec la craie neuve, puis le pain. On a entendu toute ta phrase. Un croissant jaune reste au creux de sa main. La croûte et la craie sentent le chaud, toutes les deux.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec la craie neuve, puis le pain. Tes mots sont arrivés, cette fois. Un croissant jaune reste au creux de sa main. La croûte et la craie sentent le chaud, toutes les deux.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec la craie neuve, puis le pain. On a entendu toute ta phrase. Un croissant jaune reste au creux de sa main. La croûte et la craie sentent le chaud, toutes les deux.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec la craie neuve, puis le pain. Tes mots sont arrivés, cette fois. Un croissant jaune reste au creux de sa main. La croûte et la craie sentent le chaud, toutes les deux.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -4951,7 +4951,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné sur le tapis, avec la craie neuve, puis le pain.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Un croissant jaune reste au creux de sa main.
 narrateur|La croûte et la craie sentent le chaud, toutes les deux.</t>
         </is>
@@ -4985,17 +4985,17 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Aniss lève l'ardoise vers le volet, craie au poing. Il veut finir la queue dehors. Un trait, juste un ! Le mot trop vite se perd dans le vent. Le volet bouge, le trait dérape. Aniss recule d'un pas, sur le tapis. Il attend que le bois tienne. Le volet est calme. Finis ta queue. Voilà, elle rejoint la vraie. Dehors et dedans se saluent. La boîte ronde brille sur le rebord. Sa main jaune laisse une virgule au loquet.</t>
+          <t>Aniss lève l'ardoise vers le volet, craie au poing. Il veut finir la queue dehors. Un trait, juste un ! Sa phrase trop vite se perd dans le vent. Le volet bouge, le trait dérape. Aniss recule d'un pas, sur le tapis. Il attend que le bois tienne. Le volet est calme. Finis ta queue. Voilà, elle rejoint la vraie. Dehors et dedans se saluent. La boîte ronde brille sur le rebord. Sa main jaune laisse une virgule au loquet.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss lève l'ardoise vers le volet, craie au poing. Il veut finir la queue dehors. Un trait, juste un ! Le mot trop vite se perd dans le vent. Le volet bouge, le trait dérape. Aniss recule d'un pas, sur le tapis. Il attend que le bois tienne. Le volet est calme. Finis ta queue. Voilà, elle rejoint la vraie. Dehors et dedans se saluent. La boîte ronde brille sur le rebord. Sa main jaune laisse une virgule au loquet.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss lève l'ardoise vers le volet, craie au poing. Il veut finir la queue dehors. Un trait, juste un ! Sa phrase trop vite se perd dans le vent. Le volet bouge, le trait dérape. Aniss recule d'un pas, sur le tapis. Il attend que le bois tienne. Le volet est calme. Finis ta queue. Voilà, elle rejoint la vraie. Dehors et dedans se saluent. La boîte ronde brille sur le rebord. Sa main jaune laisse une virgule au loquet.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Aniss lève l'ardoise vers le volet, craie au poing. Il veut finir la queue dehors. Un trait, juste un ! Le mot trop vite se perd dans le vent. Le volet bouge, le trait dérape. Aniss recule d'un pas, sur le tapis. Il attend que le bois tienne. Le volet est calme. Finis ta queue. Voilà, elle rejoint la vraie. Dehors et dedans se saluent. La boîte ronde brille sur le rebord. Sa main jaune laisse une virgule au loquet. [pause]</t>
+          <t>Aniss lève l'ardoise vers le volet, craie au poing. Il veut finir la queue dehors. Un trait, juste un ! Sa phrase trop vite se perd dans le vent. Le volet bouge, le trait dérape. Aniss recule d'un pas, sur le tapis. Il attend que le bois tienne. Le volet est calme. Finis ta queue. Voilà, elle rejoint la vraie. Dehors et dedans se saluent. La boîte ronde brille sur le rebord. Sa main jaune laisse une virgule au loquet. [pause]</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -5132,7 +5132,7 @@
           <t>narrateur|Aniss lève l'ardoise vers le volet, craie au poing.
 narrateur|Il veut finir la queue dehors.
 enfant-m|Un trait, juste un !
-narrateur|Le mot trop vite se perd dans le vent.
+narrateur|Sa phrase trop vite se perd dans le vent.
 narrateur|Le volet bouge, le trait dérape.
 narrateur|Aniss recule d'un pas, sur le tapis.
 narrateur|Il attend que le bois tienne.
@@ -5173,17 +5173,17 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec la craie neuve, puis le volet. On a entendu toute ta phrase. Un croissant jaune reste au creux de sa main. La boîte ronde brille sur le rebord du volet.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec la craie neuve, puis le volet. Tes mots sont arrivés, cette fois. Un croissant jaune reste au creux de sa main. La boîte ronde brille sur le rebord du volet.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec la craie neuve, puis le volet. On a entendu toute ta phrase. Un croissant jaune reste au creux de sa main. La boîte ronde brille sur le rebord du volet.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec la craie neuve, puis le volet. Tes mots sont arrivés, cette fois. Un croissant jaune reste au creux de sa main. La boîte ronde brille sur le rebord du volet.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec la craie neuve, puis le volet. On a entendu toute ta phrase. Un croissant jaune reste au creux de sa main. La boîte ronde brille sur le rebord du volet.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec la craie neuve, puis le volet. Tes mots sont arrivés, cette fois. Un croissant jaune reste au creux de sa main. La boîte ronde brille sur le rebord du volet.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -5321,7 +5321,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné sur le tapis, avec la craie neuve, puis le volet.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Un croissant jaune reste au creux de sa main.
 narrateur|La boîte ronde brille sur le rebord du volet.</t>
         </is>
@@ -5745,17 +5745,17 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Du tabouret, le clou est juste à hauteur. Aniss tend l'ardoise, les talons levés. Je l'accroche ! Papa parle, et le tabouret penche. Aniss ravalé son cri. Il attend que papa tienne le bois. Je te tiens. Vas-y, doucement. L'ardoise trouve le clou, sans choc. Il est plus grand que le tabouret. On le voit depuis le tapis. Le tabouret vide regarde trop haut. Sa main quitte le rebord, un peu fière.</t>
+          <t>Du tabouret, le clou est juste à hauteur. Aniss tend l'ardoise, les talons levés. Je l'accroche ! Papa parle, et le tabouret penche. Aniss ravale son cri. Il attend que papa tienne le bois. Je te tiens. Vas-y, doucement. L'ardoise trouve le clou, sans choc. Il est plus grand que le tabouret. On le voit depuis le tapis. Le tabouret vide regarde trop haut. Sa main quitte le rebord, un peu fière.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Du tabouret, le clou est juste à hauteur. Aniss tend l'ardoise, les talons levés. Je l'accroche ! Papa parle, et le tabouret penche. Aniss ravalé son cri. Il attend que papa tienne le bois. Je te tiens. Vas-y, doucement. L'ardoise trouve le clou, sans choc. Il est plus grand que le tabouret. On le voit depuis le tapis. Le tabouret vide regarde trop haut. Sa main quitte le rebord, un peu fière.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Du tabouret, le clou est juste à hauteur. Aniss tend l'ardoise, les talons levés. Je l'accroche ! Papa parle, et le tabouret penche. Aniss ravale son cri. Il attend que papa tienne le bois. Je te tiens. Vas-y, doucement. L'ardoise trouve le clou, sans choc. Il est plus grand que le tabouret. On le voit depuis le tapis. Le tabouret vide regarde trop haut. Sa main quitte le rebord, un peu fière.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Du tabouret, le clou est juste à hauteur. Aniss tend l'ardoise, les talons levés. Je l'accroche ! Papa parle, et le tabouret penche. Aniss ravalé son cri. Il attend que papa tienne le bois. Je te tiens. Vas-y, doucement. L'ardoise trouve le clou, sans choc. Il est plus grand que le tabouret. On le voit depuis le tapis. Le tabouret vide regarde trop haut. Sa main quitte le rebord, un peu fière. [pause]</t>
+          <t>Du tabouret, le clou est juste à hauteur. Aniss tend l'ardoise, les talons levés. Je l'accroche ! Papa parle, et le tabouret penche. Aniss ravale son cri. Il attend que papa tienne le bois. Je te tiens. Vas-y, doucement. L'ardoise trouve le clou, sans choc. Il est plus grand que le tabouret. On le voit depuis le tapis. Le tabouret vide regarde trop haut. Sa main quitte le rebord, un peu fière. [pause]</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
@@ -5893,7 +5893,7 @@
 narrateur|Aniss tend l'ardoise, les talons levés.
 enfant-m|Je l'accroche !
 narrateur|Papa parle, et le tabouret penche.
-narrateur|Aniss ravalé son cri.
+narrateur|Aniss ravale son cri.
 narrateur|Il attend que papa tienne le bois.
 papa|Je te tiens.
 papa|Vas-y, doucement.
@@ -5933,17 +5933,17 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec le tabouret, puis le clou. On a entendu toute ta phrase. Sa main sent le bois du tabouret. Le tabouret vide regarde l'ardoise, trop haute pour lui.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec le tabouret, puis le clou. Tes mots sont arrivés, cette fois. Sa main sent le bois du tabouret. Le tabouret vide regarde l'ardoise, trop haute pour lui.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec le tabouret, puis le clou. On a entendu toute ta phrase. Sa main sent le bois du tabouret. Le tabouret vide regarde l'ardoise, trop haute pour lui.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec le tabouret, puis le clou. Tes mots sont arrivés, cette fois. Sa main sent le bois du tabouret. Le tabouret vide regarde l'ardoise, trop haute pour lui.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec le tabouret, puis le clou. On a entendu toute ta phrase. Sa main sent le bois du tabouret. Le tabouret vide regarde l'ardoise, trop haute pour lui.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec le tabouret, puis le clou. Tes mots sont arrivés, cette fois. Sa main sent le bois du tabouret. Le tabouret vide regarde l'ardoise, trop haute pour lui.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -6081,7 +6081,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné sur le tapis, avec le tabouret, puis le clou.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Sa main sent le bois du tabouret.
 narrateur|Le tabouret vide regarde l'ardoise, trop haute pour lui.</t>
         </is>
@@ -6303,17 +6303,17 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec le tabouret, puis le pain. On a entendu toute ta phrase. Sa main sent le bois du tabouret. Aniss redescend ; le pain et l'ardoise partagent le soleil.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec le tabouret, puis le pain. Tes mots sont arrivés, cette fois. Sa main sent le bois du tabouret. Aniss redescend ; le pain et l'ardoise partagent le soleil.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec le tabouret, puis le pain. On a entendu toute ta phrase. Sa main sent le bois du tabouret. Aniss redescend ; le pain et l'ardoise partagent le soleil.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec le tabouret, puis le pain. Tes mots sont arrivés, cette fois. Sa main sent le bois du tabouret. Aniss redescend ; le pain et l'ardoise partagent le soleil.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec le tabouret, puis le pain. On a entendu toute ta phrase. Sa main sent le bois du tabouret. Aniss redescend ; le pain et l'ardoise partagent le soleil.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec le tabouret, puis le pain. Tes mots sont arrivés, cette fois. Sa main sent le bois du tabouret. Aniss redescend ; le pain et l'ardoise partagent le soleil.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -6451,7 +6451,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné sur le tapis, avec le tabouret, puis le pain.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Sa main sent le bois du tabouret.
 narrateur|Aniss redescend ; le pain et l'ardoise partagent le soleil.</t>
         </is>
@@ -6485,17 +6485,17 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Aniss, sur le tabouret, attrape le volet. Il veut coller l'ardoise au bois. Regarde, c'est le même ! Le vent répond à sa place. Le volet frappe, presque. Aniss se tait, une main sur le loquet. Je retiens le bois. Parle, maintenant. Dehors il danse, ici il tient. Deux danses, une seule histoire de queue. Sa main haute garde le volet. Le tabouret ne bouge plus. Un fil de laine s'accroche à son talon.</t>
+          <t>Aniss, sur le tabouret, attrape le volet. Il veut coller l'ardoise au bois. Regarde, c'est le même ! Le vent répond à sa place. Le volet frappe, presque. Aniss se tait, une main sur le loquet. Je retiens le bois. Parle, maintenant. Dehors il danse, ici il tient. Deux danses, et une seule queue. Sa main haute garde le volet. Le tabouret ne bouge plus. Un fil de laine s'accroche à son talon.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss, sur le tabouret, attrape le volet. Il veut coller l'ardoise au bois. Regarde, c'est le même ! Le vent répond à sa place. Le volet frappe, presque. Aniss se tait, une main sur le loquet. Je retiens le bois. Parle, maintenant. Dehors il danse, ici il tient. Deux danses, une seule histoire de queue. Sa main haute garde le volet. Le tabouret ne bouge plus. Un fil de laine s'accroche à son talon.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss, sur le tabouret, attrape le volet. Il veut coller l'ardoise au bois. Regarde, c'est le même ! Le vent répond à sa place. Le volet frappe, presque. Aniss se tait, une main sur le loquet. Je retiens le bois. Parle, maintenant. Dehors il danse, ici il tient. Deux danses, et une seule queue. Sa main haute garde le volet. Le tabouret ne bouge plus. Un fil de laine s'accroche à son talon.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Aniss, sur le tabouret, attrape le volet. Il veut coller l'ardoise au bois. Regarde, c'est le même ! Le vent répond à sa place. Le volet frappe, presque. Aniss se tait, une main sur le loquet. Je retiens le bois. Parle, maintenant. Dehors il danse, ici il tient. Deux danses, une seule histoire de queue. Sa main haute garde le volet. Le tabouret ne bouge plus. Un fil de laine s'accroche à son talon. [pause]</t>
+          <t>Aniss, sur le tabouret, attrape le volet. Il veut coller l'ardoise au bois. Regarde, c'est le même ! Le vent répond à sa place. Le volet frappe, presque. Aniss se tait, une main sur le loquet. Je retiens le bois. Parle, maintenant. Dehors il danse, ici il tient. Deux danses, et une seule queue. Sa main haute garde le volet. Le tabouret ne bouge plus. Un fil de laine s'accroche à son talon. [pause]</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -6638,7 +6638,7 @@
 papa|Je retiens le bois.
 papa|Parle, maintenant.
 enfant-m|Dehors il danse, ici il tient.
-maman|Deux danses, une seule histoire de queue.
+maman|Deux danses, et une seule queue.
 narrateur|Sa main haute garde le volet.
 narrateur|Le tabouret ne bouge plus.
 narrateur|Un fil de laine s'accroche à son talon.</t>
@@ -6673,17 +6673,17 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec le tabouret, puis le volet. On a entendu toute ta phrase. Sa main sent le bois du tabouret. Sa main tient le volet, sans bouger, là-haut.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec le tabouret, puis le volet. Tes mots sont arrivés, cette fois. Sa main sent le bois du tabouret. Sa main tient le volet, sans bouger, là-haut.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec le tabouret, puis le volet. On a entendu toute ta phrase. Sa main sent le bois du tabouret. Sa main tient le volet, sans bouger, là-haut.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec le tabouret, puis le volet. Tes mots sont arrivés, cette fois. Sa main sent le bois du tabouret. Sa main tient le volet, sans bouger, là-haut.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec le tabouret, puis le volet. On a entendu toute ta phrase. Sa main sent le bois du tabouret. Sa main tient le volet, sans bouger, là-haut.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur le tapis, avec le tabouret, puis le volet. Tes mots sont arrivés, cette fois. Sa main sent le bois du tabouret. Sa main tient le volet, sans bouger, là-haut.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -6821,7 +6821,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné sur le tapis, avec le tabouret, puis le volet.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Sa main sent le bois du tabouret.
 narrateur|Sa main tient le volet, sans bouger, là-haut.</t>
         </is>
@@ -8190,17 +8190,17 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec l'éponge, puis le clou. On a entendu toute ta phrase. Ses doigts sentent l'eau et la farine. Des miettes collent au bord mouillé de l'ardoise.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec l'éponge, puis le clou. Tes mots sont arrivés, cette fois. Ses doigts sentent l'eau et la farine. Des miettes collent au bord mouillé de l'ardoise.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec l'éponge, puis le clou. On a entendu toute ta phrase. Ses doigts sentent l'eau et la farine. Des miettes collent au bord mouillé de l'ardoise.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec l'éponge, puis le clou. Tes mots sont arrivés, cette fois. Ses doigts sentent l'eau et la farine. Des miettes collent au bord mouillé de l'ardoise.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec l'éponge, puis le clou. On a entendu toute ta phrase. Ses doigts sentent l'eau et la farine. Des miettes collent au bord mouillé de l'ardoise.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec l'éponge, puis le clou. Tes mots sont arrivés, cette fois. Ses doigts sentent l'eau et la farine. Des miettes collent au bord mouillé de l'ardoise.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
@@ -8338,7 +8338,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné sur la table, avec l'éponge, puis le clou.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Ses doigts sentent l'eau et la farine.
 narrateur|Des miettes collent au bord mouillé de l'ardoise.</t>
         </is>
@@ -8560,17 +8560,17 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec l'éponge, puis le pain. On a entendu toute ta phrase. Ses doigts sentent l'eau et la farine. Le couteau repose ; le cerf-volant pâle sèche au pain.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec l'éponge, puis le pain. Tes mots sont arrivés, cette fois. Ses doigts sentent l'eau et la farine. Le couteau repose ; le cerf-volant pâle sèche au pain.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec l'éponge, puis le pain. On a entendu toute ta phrase. Ses doigts sentent l'eau et la farine. Le couteau repose ; le cerf-volant pâle sèche au pain.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec l'éponge, puis le pain. Tes mots sont arrivés, cette fois. Ses doigts sentent l'eau et la farine. Le couteau repose ; le cerf-volant pâle sèche au pain.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec l'éponge, puis le pain. On a entendu toute ta phrase. Ses doigts sentent l'eau et la farine. Le couteau repose ; le cerf-volant pâle sèche au pain.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec l'éponge, puis le pain. Tes mots sont arrivés, cette fois. Ses doigts sentent l'eau et la farine. Le couteau repose ; le cerf-volant pâle sèche au pain.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
@@ -8708,7 +8708,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné sur la table, avec l'éponge, puis le pain.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Ses doigts sentent l'eau et la farine.
 narrateur|Le couteau repose ; le cerf-volant pâle sèche au pain.</t>
         </is>
@@ -8742,17 +8742,17 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Aniss pousse l'ardoise mouillée vers le volet. Une goutte court sur la table, vers les pièces. Vite, le vrai est là ! Les pièces tintent, papa répond. La goutte s'arrête contre une pièce. Aniss retient sa phrase. Les pièces sont sages. Ouvre le volet, on compare. Pâle ici, rouge là-bas. Deux versions, une même queue. L'éponge laisse un rond sur le bois. Sa main écarte le volet, sans claquer. Le figuier entre dans la cuisine.</t>
+          <t>Aniss pousse l'ardoise mouillée vers le volet. Une goutte court sur la table, vers les pièces. Vite, le vrai est là ! Les pièces tintent, papa répond. La goutte s'arrête contre une pièce. Aniss retient sa phrase. Les pièces sont sages. Ouvre le volet, on compare. Pâle ici, rouge là-bas. Deux queues, une pâle, une rouge. L'éponge laisse un rond sur le bois. Sa main écarte le volet, sans claquer. Le figuier entre dans la cuisine.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss pousse l'ardoise mouillée vers le volet. Une goutte court sur la table, vers les pièces. Vite, le vrai est là ! Les pièces tintent, papa répond. La goutte s'arrête contre une pièce. Aniss retient sa phrase. Les pièces sont sages. Ouvre le volet, on compare. Pâle ici, rouge là-bas. Deux versions, une même queue. L'éponge laisse un rond sur le bois. Sa main écarte le volet, sans claquer. Le figuier entre dans la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss pousse l'ardoise mouillée vers le volet. Une goutte court sur la table, vers les pièces. Vite, le vrai est là ! Les pièces tintent, papa répond. La goutte s'arrête contre une pièce. Aniss retient sa phrase. Les pièces sont sages. Ouvre le volet, on compare. Pâle ici, rouge là-bas. Deux queues, une pâle, une rouge. L'éponge laisse un rond sur le bois. Sa main écarte le volet, sans claquer. Le figuier entre dans la cuisine.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Aniss pousse l'ardoise mouillée vers le volet. Une goutte court sur la table, vers les pièces. Vite, le vrai est là ! Les pièces tintent, papa répond. La goutte s'arrête contre une pièce. Aniss retient sa phrase. Les pièces sont sages. Ouvre le volet, on compare. Pâle ici, rouge là-bas. Deux versions, une même queue. L'éponge laisse un rond sur le bois. Sa main écarte le volet, sans claquer. Le figuier entre dans la cuisine. [pause]</t>
+          <t>Aniss pousse l'ardoise mouillée vers le volet. Une goutte court sur la table, vers les pièces. Vite, le vrai est là ! Les pièces tintent, papa répond. La goutte s'arrête contre une pièce. Aniss retient sa phrase. Les pièces sont sages. Ouvre le volet, on compare. Pâle ici, rouge là-bas. Deux queues, une pâle, une rouge. L'éponge laisse un rond sur le bois. Sa main écarte le volet, sans claquer. Le figuier entre dans la cuisine. [pause]</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
@@ -8895,7 +8895,7 @@
 papa|Les pièces sont sages.
 papa|Ouvre le volet, on compare.
 enfant-m|Pâle ici, rouge là-bas.
-maman|Deux versions, une même queue.
+maman|Deux queues, une pâle, une rouge.
 narrateur|L'éponge laisse un rond sur le bois.
 narrateur|Sa main écarte le volet, sans claquer.
 narrateur|Le figuier entre dans la cuisine.</t>
@@ -8930,17 +8930,17 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec l'éponge, puis le volet. On a entendu toute ta phrase. Ses doigts sentent l'eau et la farine. Une goutte court vers les pièces, puis s'arrête.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec l'éponge, puis le volet. Tes mots sont arrivés, cette fois. Ses doigts sentent l'eau et la farine. Une goutte court vers les pièces, puis s'arrête.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec l'éponge, puis le volet. On a entendu toute ta phrase. Ses doigts sentent l'eau et la farine. Une goutte court vers les pièces, puis s'arrête.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec l'éponge, puis le volet. Tes mots sont arrivés, cette fois. Ses doigts sentent l'eau et la farine. Une goutte court vers les pièces, puis s'arrête.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec l'éponge, puis le volet. On a entendu toute ta phrase. Ses doigts sentent l'eau et la farine. Une goutte court vers les pièces, puis s'arrête.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec l'éponge, puis le volet. Tes mots sont arrivés, cette fois. Ses doigts sentent l'eau et la farine. Une goutte court vers les pièces, puis s'arrête.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -9078,7 +9078,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné sur la table, avec l'éponge, puis le volet.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Ses doigts sentent l'eau et la farine.
 narrateur|Une goutte court vers les pièces, puis s'arrête.</t>
         </is>
@@ -9690,17 +9690,17 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec la craie neuve, puis le clou. On a entendu toute ta phrase. Deux poudres blanches ornent ses ongles. La boîte ronde garde le pied du clou.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec la craie neuve, puis le clou. Tes mots sont arrivés, cette fois. Deux poudres blanches ornent ses ongles. La boîte ronde garde le pied du clou.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec la craie neuve, puis le clou. On a entendu toute ta phrase. Deux poudres blanches ornent ses ongles. La boîte ronde garde le pied du clou.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec la craie neuve, puis le clou. Tes mots sont arrivés, cette fois. Deux poudres blanches ornent ses ongles. La boîte ronde garde le pied du clou.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec la craie neuve, puis le clou. On a entendu toute ta phrase. Deux poudres blanches ornent ses ongles. La boîte ronde garde le pied du clou.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec la craie neuve, puis le clou. Tes mots sont arrivés, cette fois. Deux poudres blanches ornent ses ongles. La boîte ronde garde le pied du clou.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -9838,7 +9838,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné sur la table, avec la craie neuve, puis le clou.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Deux poudres blanches ornent ses ongles.
 narrateur|La boîte ronde garde le pied du clou.</t>
         </is>
@@ -10060,17 +10060,17 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec la craie neuve, puis le pain. On a entendu toute ta phrase. Deux poudres blanches ornent ses ongles. Farine et craie se mêlent au bout de ses doigts.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec la craie neuve, puis le pain. Tes mots sont arrivés, cette fois. Deux poudres blanches ornent ses ongles. Farine et craie se mêlent au bout de ses doigts.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec la craie neuve, puis le pain. On a entendu toute ta phrase. Deux poudres blanches ornent ses ongles. Farine et craie se mêlent au bout de ses doigts.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec la craie neuve, puis le pain. Tes mots sont arrivés, cette fois. Deux poudres blanches ornent ses ongles. Farine et craie se mêlent au bout de ses doigts.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec la craie neuve, puis le pain. On a entendu toute ta phrase. Deux poudres blanches ornent ses ongles. Farine et craie se mêlent au bout de ses doigts.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec la craie neuve, puis le pain. Tes mots sont arrivés, cette fois. Deux poudres blanches ornent ses ongles. Farine et craie se mêlent au bout de ses doigts.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -10208,7 +10208,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné sur la table, avec la craie neuve, puis le pain.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Deux poudres blanches ornent ses ongles.
 narrateur|Farine et craie se mêlent au bout de ses doigts.</t>
         </is>
@@ -10242,17 +10242,17 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Aniss porte craie et ardoise vers le volet. Il veut la dernière ligne pendant que papa parle. La nervure de la feuille ! Le volet cède d'un souffle. La ligne part de travers. Aniss pose la craie, les lèvres closes. Je tiens le volet. Recommence la nervure. Voilà, elle rejoint le figuier. Le volet dort, la ligne est nette. Un grain jaune reste au loquet. Sa main ne cache plus le dessin. Dehors, le rouge approuve, sans un mot.</t>
+          <t>Aniss porte craie et ardoise vers le volet. Il veut la dernière ligne pendant que papa parle. Le trait de la feuille ! Le volet cède d'un souffle. La ligne part de travers. Aniss pose la craie, les lèvres closes. Je tiens le volet. Recommence le trait de feuille. Voilà, elle rejoint le figuier. Le volet dort, la ligne est nette. Un grain jaune reste au loquet. Sa main ne cache plus le dessin. Dehors, le rouge approuve, sans un mot.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss porte craie et ardoise vers le volet. Il veut la dernière ligne pendant que papa parle. La nervure de la feuille ! Le volet cède d'un souffle. La ligne part de travers. Aniss pose la craie, les lèvres closes. Je tiens le volet. Recommence la nervure. Voilà, elle rejoint le figuier. Le volet dort, la ligne est nette. Un grain jaune reste au loquet. Sa main ne cache plus le dessin. Dehors, le rouge approuve, sans un mot.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss porte craie et ardoise vers le volet. Il veut la dernière ligne pendant que papa parle. Le trait de la feuille ! Le volet cède d'un souffle. La ligne part de travers. Aniss pose la craie, les lèvres closes. Je tiens le volet. Recommence le trait de feuille. Voilà, elle rejoint le figuier. Le volet dort, la ligne est nette. Un grain jaune reste au loquet. Sa main ne cache plus le dessin. Dehors, le rouge approuve, sans un mot.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Aniss porte craie et ardoise vers le volet. Il veut la dernière ligne pendant que papa parle. La nervure de la feuille ! Le volet cède d'un souffle. La ligne part de travers. Aniss pose la craie, les lèvres closes. Je tiens le volet. Recommence la nervure. Voilà, elle rejoint le figuier. Le volet dort, la ligne est nette. Un grain jaune reste au loquet. Sa main ne cache plus le dessin. Dehors, le rouge approuve, sans un mot. [pause]</t>
+          <t>Aniss porte craie et ardoise vers le volet. Il veut la dernière ligne pendant que papa parle. Le trait de la feuille ! Le volet cède d'un souffle. La ligne part de travers. Aniss pose la craie, les lèvres closes. Je tiens le volet. Recommence le trait de feuille. Voilà, elle rejoint le figuier. Le volet dort, la ligne est nette. Un grain jaune reste au loquet. Sa main ne cache plus le dessin. Dehors, le rouge approuve, sans un mot. [pause]</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -10388,12 +10388,12 @@
         <is>
           <t>narrateur|Aniss porte craie et ardoise vers le volet.
 narrateur|Il veut la dernière ligne pendant que papa parle.
-enfant-m|La nervure de la feuille !
+enfant-m|Le trait de la feuille !
 narrateur|Le volet cède d'un souffle.
 narrateur|La ligne part de travers.
 narrateur|Aniss pose la craie, les lèvres closes.
 papa|Je tiens le volet.
-papa|Recommence la nervure.
+papa|Recommence le trait de feuille.
 enfant-m|Voilà, elle rejoint le figuier.
 maman|Le volet dort, la ligne est nette.
 narrateur|Un grain jaune reste au loquet.
@@ -10430,17 +10430,17 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec la craie neuve, puis le volet. On a entendu toute ta phrase. Deux poudres blanches ornent ses ongles. Le volet dort ; la dernière ligne est nette.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec la craie neuve, puis le volet. Tes mots sont arrivés, cette fois. Deux poudres blanches ornent ses ongles. Le volet dort ; la dernière ligne est nette.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec la craie neuve, puis le volet. On a entendu toute ta phrase. Deux poudres blanches ornent ses ongles. Le volet dort ; la dernière ligne est nette.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec la craie neuve, puis le volet. Tes mots sont arrivés, cette fois. Deux poudres blanches ornent ses ongles. Le volet dort ; la dernière ligne est nette.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec la craie neuve, puis le volet. On a entendu toute ta phrase. Deux poudres blanches ornent ses ongles. Le volet dort ; la dernière ligne est nette.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec la craie neuve, puis le volet. Tes mots sont arrivés, cette fois. Deux poudres blanches ornent ses ongles. Le volet dort ; la dernière ligne est nette.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
@@ -10578,7 +10578,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné sur la table, avec la craie neuve, puis le volet.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Deux poudres blanches ornent ses ongles.
 narrateur|Le volet dort ; la dernière ligne est nette.</t>
         </is>
@@ -11002,17 +11002,17 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Aniss pousse le tabouret sous le clou. La table recule d'un doigt. Je le mets en haut ! Une cuillère tombe, et papa s'exclame. Les mots d'Aniss se cassent. Il attend que la cuillère se taise. C'est bon, j'ai ramassé. Monte. L'ardoise gagne le clou, au-dessus du pain. Il surveille la table. Le tabouret rentre, l'ardoise veille. Sa main quitte le bois, un peu blanche. Une miette orpheline reste sur une barre.</t>
+          <t>Aniss pousse le tabouret sous le clou. La table recule d'un doigt. Je le mets en haut ! Une cuillère tombe, et papa s'exclame. Les mots d'Aniss se cassent. Il attend que la cuillère se taise. C'est bon, j'ai ramassé. Monte. L'ardoise gagne le clou, au-dessus du pain. Il surveille la table. Le tabouret rentre, l'ardoise veille. Sa main quitte le bois, un peu blanche. Une miette oubliée reste sur une barre.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss pousse le tabouret sous le clou. La table recule d'un doigt. Je le mets en haut ! Une cuillère tombe, et papa s'exclame. Les mots d'Aniss se cassent. Il attend que la cuillère se taise. C'est bon, j'ai ramassé. Monte. L'ardoise gagne le clou, au-dessus du pain. Il surveille la table. Le tabouret rentre, l'ardoise veille. Sa main quitte le bois, un peu blanche. Une miette orpheline reste sur une barre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss pousse le tabouret sous le clou. La table recule d'un doigt. Je le mets en haut ! Une cuillère tombe, et papa s'exclame. Les mots d'Aniss se cassent. Il attend que la cuillère se taise. C'est bon, j'ai ramassé. Monte. L'ardoise gagne le clou, au-dessus du pain. Il surveille la table. Le tabouret rentre, l'ardoise veille. Sa main quitte le bois, un peu blanche. Une miette oubliée reste sur une barre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Aniss pousse le tabouret sous le clou. La table recule d'un doigt. Je le mets en haut ! Une cuillère tombe, et papa s'exclame. Les mots d'Aniss se cassent. Il attend que la cuillère se taise. C'est bon, j'ai ramassé. Monte. L'ardoise gagne le clou, au-dessus du pain. Il surveille la table. Le tabouret rentre, l'ardoise veille. Sa main quitte le bois, un peu blanche. Une miette orpheline reste sur une barre. [pause]</t>
+          <t>Aniss pousse le tabouret sous le clou. La table recule d'un doigt. Je le mets en haut ! Une cuillère tombe, et papa s'exclame. Les mots d'Aniss se cassent. Il attend que la cuillère se taise. C'est bon, j'ai ramassé. Monte. L'ardoise gagne le clou, au-dessus du pain. Il surveille la table. Le tabouret rentre, l'ardoise veille. Sa main quitte le bois, un peu blanche. Une miette oubliée reste sur une barre. [pause]</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -11158,7 +11158,7 @@
 enfant-m|Il surveille la table.
 maman|Le tabouret rentre, l'ardoise veille.
 narrateur|Sa main quitte le bois, un peu blanche.
-narrateur|Une miette orpheline reste sur une barre.</t>
+narrateur|Une miette oubliée reste sur une barre.</t>
         </is>
       </c>
       <c r="AX54" t="inlineStr">
@@ -11190,17 +11190,17 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec le tabouret, puis le clou. On a entendu toute ta phrase. Sa main a gardé la chaleur de la nappe. Le tabouret rentre sous la table ; l'ardoise veille.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec le tabouret, puis le clou. Tes mots sont arrivés, cette fois. Sa main a gardé la chaleur de la nappe. Le tabouret rentre sous la table ; l'ardoise veille.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec le tabouret, puis le clou. On a entendu toute ta phrase. Sa main a gardé la chaleur de la nappe. Le tabouret rentre sous la table ; l'ardoise veille.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec le tabouret, puis le clou. Tes mots sont arrivés, cette fois. Sa main a gardé la chaleur de la nappe. Le tabouret rentre sous la table ; l'ardoise veille.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec le tabouret, puis le clou. On a entendu toute ta phrase. Sa main a gardé la chaleur de la nappe. Le tabouret rentre sous la table ; l'ardoise veille.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec le tabouret, puis le clou. Tes mots sont arrivés, cette fois. Sa main a gardé la chaleur de la nappe. Le tabouret rentre sous la table ; l'ardoise veille.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -11338,7 +11338,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné sur la table, avec le tabouret, puis le clou.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Sa main a gardé la chaleur de la nappe.
 narrateur|Le tabouret rentre sous la table ; l'ardoise veille.</t>
         </is>
@@ -11560,17 +11560,17 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec le tabouret, puis le pain. On a entendu toute ta phrase. Sa main a gardé la chaleur de la nappe. Le cerf-volant de craie fait face à la miche.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec le tabouret, puis le pain. Tes mots sont arrivés, cette fois. Sa main a gardé la chaleur de la nappe. Le cerf-volant de craie fait face à la miche.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec le tabouret, puis le pain. On a entendu toute ta phrase. Sa main a gardé la chaleur de la nappe. Le cerf-volant de craie fait face à la miche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec le tabouret, puis le pain. Tes mots sont arrivés, cette fois. Sa main a gardé la chaleur de la nappe. Le cerf-volant de craie fait face à la miche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec le tabouret, puis le pain. On a entendu toute ta phrase. Sa main a gardé la chaleur de la nappe. Le cerf-volant de craie fait face à la miche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec le tabouret, puis le pain. Tes mots sont arrivés, cette fois. Sa main a gardé la chaleur de la nappe. Le cerf-volant de craie fait face à la miche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
@@ -11708,7 +11708,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné sur la table, avec le tabouret, puis le pain.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Sa main a gardé la chaleur de la nappe.
 narrateur|Le cerf-volant de craie fait face à la miche.</t>
         </is>
@@ -11742,17 +11742,17 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Aniss hisse le tabouret contre le volet. Du haut, le figuier remplit la vitre. Il est énorme ! Papa veut fermer un peu, à cause du soleil. Leurs envies se croisent. Aniss pose l'ardoise, et il attend. On laisse ouvert ? Oui, pour copier la grande queue. Alors on compare, sans bouger le bois. Le cerf-volant de craie salue le vrai. Du tabouret, la place entière tient dans un cadre. Sa main ombre un coin de l'ardoise. On voit tout, grâce à toi.</t>
+          <t>Aniss pousse le tabouret contre le volet. Du haut, le figuier remplit la vitre. Il est énorme ! Papa veut fermer un peu, à cause du soleil. Leurs envies se croisent. Aniss pose l'ardoise, et il attend. On laisse ouvert ? Oui, pour copier la grande queue. Alors on compare, sans bouger le bois. Le cerf-volant de craie salue le vrai. Du tabouret, la place entière tient dans un cadre. Sa main ombre un coin de l'ardoise. On voit tout, grâce à toi.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss hisse le tabouret contre le volet. Du haut, le figuier remplit la vitre. Il est énorme ! Papa veut fermer un peu, à cause du soleil. Leurs envies se croisent. Aniss pose l'ardoise, et il attend. On laisse ouvert ? Oui, pour copier la grande queue. Alors on compare, sans bouger le bois. Le cerf-volant de craie salue le vrai. Du tabouret, la place entière tient dans un cadre. Sa main ombre un coin de l'ardoise. On voit tout, grâce à toi.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss pousse le tabouret contre le volet. Du haut, le figuier remplit la vitre. Il est énorme ! Papa veut fermer un peu, à cause du soleil. Leurs envies se croisent. Aniss pose l'ardoise, et il attend. On laisse ouvert ? Oui, pour copier la grande queue. Alors on compare, sans bouger le bois. Le cerf-volant de craie salue le vrai. Du tabouret, la place entière tient dans un cadre. Sa main ombre un coin de l'ardoise. On voit tout, grâce à toi.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Aniss hisse le tabouret contre le volet. Du haut, le figuier remplit la vitre. Il est énorme ! Papa veut fermer un peu, à cause du soleil. Leurs envies se croisent. Aniss pose l'ardoise, et il attend. On laisse ouvert ? Oui, pour copier la grande queue. Alors on compare, sans bouger le bois. Le cerf-volant de craie salue le vrai. Du tabouret, la place entière tient dans un cadre. Sa main ombre un coin de l'ardoise. On voit tout, grâce à toi. [pause]</t>
+          <t>Aniss pousse le tabouret contre le volet. Du haut, le figuier remplit la vitre. Il est énorme ! Papa veut fermer un peu, à cause du soleil. Leurs envies se croisent. Aniss pose l'ardoise, et il attend. On laisse ouvert ? Oui, pour copier la grande queue. Alors on compare, sans bouger le bois. Le cerf-volant de craie salue le vrai. Du tabouret, la place entière tient dans un cadre. Sa main ombre un coin de l'ardoise. On voit tout, grâce à toi. [pause]</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -11886,7 +11886,7 @@
       </c>
       <c r="AW58" t="inlineStr">
         <is>
-          <t>narrateur|Aniss hisse le tabouret contre le volet.
+          <t>narrateur|Aniss pousse le tabouret contre le volet.
 narrateur|Du haut, le figuier remplit la vitre.
 enfant-m|Il est énorme !
 narrateur|Papa veut fermer un peu, à cause du soleil.
@@ -11930,17 +11930,17 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec le tabouret, puis le volet. On a entendu toute ta phrase. Sa main a gardé la chaleur de la nappe. Du tabouret, le figuier remplit toute la vitre.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec le tabouret, puis le volet. Tes mots sont arrivés, cette fois. Sa main a gardé la chaleur de la nappe. Du tabouret, le figuier remplit toute la vitre.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec le tabouret, puis le volet. On a entendu toute ta phrase. Sa main a gardé la chaleur de la nappe. Du tabouret, le figuier remplit toute la vitre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec le tabouret, puis le volet. Tes mots sont arrivés, cette fois. Sa main a gardé la chaleur de la nappe. Du tabouret, le figuier remplit toute la vitre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec le tabouret, puis le volet. On a entendu toute ta phrase. Sa main a gardé la chaleur de la nappe. Du tabouret, le figuier remplit toute la vitre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné sur la table, avec le tabouret, puis le volet. Tes mots sont arrivés, cette fois. Sa main a gardé la chaleur de la nappe. Du tabouret, le figuier remplit toute la vitre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
@@ -12078,7 +12078,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné sur la table, avec le tabouret, puis le volet.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Sa main a gardé la chaleur de la nappe.
 narrateur|Du tabouret, le figuier remplit toute la vitre.</t>
         </is>
@@ -13259,17 +13259,17 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>L'ardoise fraîche veut le clou, près de la vitre. Aniss marche trop vite, l'éponge sous le bras. Je le mets ici, pile ! Maman cherche ses mots sur le loquet. Une goutte file vers le rebord. Aniss s'arrête, talons au sol. Le clou est à toi. Le triangle pâle se pend, un peu froid. Les feuilles tapent, contre le verre. Elles applaudissent, peut-être. L'éponge reste sur le rebord, en sentinelle. Sa main laisse un croissant d'eau sous le clou. On le verra, chaque fois qu'on ouvre.</t>
+          <t>L'ardoise fraîche veut le clou, près de la vitre. Aniss marche trop vite, l'éponge sous le bras. Je le mets ici, pile ! Maman cherche ses mots sur le loquet. Une goutte file vers le rebord. Aniss s'arrête, talons au sol. Le clou est à toi. Le triangle pâle se pend, un peu froid. Les feuilles tapent, contre le verre. Elles applaudissent, peut-être. L'éponge reste sur le rebord, comme une garde. Sa main laisse un croissant d'eau sous le clou. On le verra, chaque fois qu'on ouvre.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;L'ardoise fraîche veut le clou, près de la vitre. Aniss marche trop vite, l'éponge sous le bras. Je le mets ici, pile ! Maman cherche ses mots sur le loquet. Une goutte file vers le rebord. Aniss s'arrête, talons au sol. Le clou est à toi. Le triangle pâle se pend, un peu froid. Les feuilles tapent, contre le verre. Elles applaudissent, peut-être. L'éponge reste sur le rebord, en sentinelle. Sa main laisse un croissant d'eau sous le clou. On le verra, chaque fois qu'on ouvre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;L'ardoise fraîche veut le clou, près de la vitre. Aniss marche trop vite, l'éponge sous le bras. Je le mets ici, pile ! Maman cherche ses mots sur le loquet. Une goutte file vers le rebord. Aniss s'arrête, talons au sol. Le clou est à toi. Le triangle pâle se pend, un peu froid. Les feuilles tapent, contre le verre. Elles applaudissent, peut-être. L'éponge reste sur le rebord, comme une garde. Sa main laisse un croissant d'eau sous le clou. On le verra, chaque fois qu'on ouvre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>L'ardoise fraîche veut le clou, près de la vitre. Aniss marche trop vite, l'éponge sous le bras. Je le mets ici, pile ! Maman cherche ses mots sur le loquet. Une goutte file vers le rebord. Aniss s'arrête, talons au sol. Le clou est à toi. Le triangle pâle se pend, un peu froid. Les feuilles tapent, contre le verre. Elles applaudissent, peut-être. L'éponge reste sur le rebord, en sentinelle. Sa main laisse un croissant d'eau sous le clou. On le verra, chaque fois qu'on ouvre. [pause]</t>
+          <t>L'ardoise fraîche veut le clou, près de la vitre. Aniss marche trop vite, l'éponge sous le bras. Je le mets ici, pile ! Maman cherche ses mots sur le loquet. Une goutte file vers le rebord. Aniss s'arrête, talons au sol. Le clou est à toi. Le triangle pâle se pend, un peu froid. Les feuilles tapent, contre le verre. Elles applaudissent, peut-être. L'éponge reste sur le rebord, comme une garde. Sa main laisse un croissant d'eau sous le clou. On le verra, chaque fois qu'on ouvre. [pause]</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -13413,7 +13413,7 @@
 narrateur|Le triangle pâle se pend, un peu froid.
 enfant-m|Les feuilles tapent, contre le verre.
 papa|Elles applaudissent, peut-être.
-narrateur|L'éponge reste sur le rebord, en sentinelle.
+narrateur|L'éponge reste sur le rebord, comme une garde.
 narrateur|Sa main laisse un croissant d'eau sous le clou.
 maman|On le verra, chaque fois qu'on ouvre.</t>
         </is>
@@ -13447,17 +13447,17 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec l'éponge, puis le clou. On a entendu toute ta phrase. Sa main sent le rebord, et un peu d'eau. Les feuilles du figuier tapent la vitre, contre l'ardoise.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec l'éponge, puis le clou. Tes mots sont arrivés, cette fois. Sa main sent le rebord, et un peu d'eau. Les feuilles du figuier tapent la vitre, contre l'ardoise.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec l'éponge, puis le clou. On a entendu toute ta phrase. Sa main sent le rebord, et un peu d'eau. Les feuilles du figuier tapent la vitre, contre l'ardoise.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec l'éponge, puis le clou. Tes mots sont arrivés, cette fois. Sa main sent le rebord, et un peu d'eau. Les feuilles du figuier tapent la vitre, contre l'ardoise.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec l'éponge, puis le clou. On a entendu toute ta phrase. Sa main sent le rebord, et un peu d'eau. Les feuilles du figuier tapent la vitre, contre l'ardoise.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec l'éponge, puis le clou. Tes mots sont arrivés, cette fois. Sa main sent le rebord, et un peu d'eau. Les feuilles du figuier tapent la vitre, contre l'ardoise.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr"/>
@@ -13595,7 +13595,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné près de la fenêtre, avec l'éponge, puis le clou.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Sa main sent le rebord, et un peu d'eau.
 narrateur|Les feuilles du figuier tapent la vitre, contre l'ardoise.</t>
         </is>
@@ -13629,17 +13629,17 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Aniss apporte l'ardoise mouillée vers le pain, à la fenêtre. Le rebord est étroit. On mange avec lui ! Papa pose deux tasses, et compte à voix haute. L'ardoise glisse d'un souffle. Aniss la plaque, sans parler. Il attend la deuxième tasse. Voilà, c'est posé. Ton dessin peut s'asseoir. Il sèche au soleil du pain. On croque, et lui sèche. Une goutte meurt sur la croûte, minuscule. Sa main sent le tiède du rebord.</t>
+          <t>Aniss apporte l'ardoise mouillée vers le pain, à la fenêtre. Le rebord est étroit. On mange avec lui ! Papa pose deux tasses, et compte à voix haute. L'ardoise glisse d'un souffle. Aniss la retient, sans parler. Il attend la deuxième tasse. Voilà, c'est posé. Ton dessin peut s'asseoir. Il sèche au soleil du pain. On croque, et lui sèche. Une goutte meurt sur la croûte, minuscule. Sa main sent le tiède du rebord.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss apporte l'ardoise mouillée vers le pain, à la fenêtre. Le rebord est étroit. On mange avec lui ! Papa pose deux tasses, et compte à voix haute. L'ardoise glisse d'un souffle. Aniss la plaque, sans parler. Il attend la deuxième tasse. Voilà, c'est posé. Ton dessin peut s'asseoir. Il sèche au soleil du pain. On croque, et lui sèche. Une goutte meurt sur la croûte, minuscule. Sa main sent le tiède du rebord.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss apporte l'ardoise mouillée vers le pain, à la fenêtre. Le rebord est étroit. On mange avec lui ! Papa pose deux tasses, et compte à voix haute. L'ardoise glisse d'un souffle. Aniss la retient, sans parler. Il attend la deuxième tasse. Voilà, c'est posé. Ton dessin peut s'asseoir. Il sèche au soleil du pain. On croque, et lui sèche. Une goutte meurt sur la croûte, minuscule. Sa main sent le tiède du rebord.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Aniss apporte l'ardoise mouillée vers le pain, à la fenêtre. Le rebord est étroit. On mange avec lui ! Papa pose deux tasses, et compte à voix haute. L'ardoise glisse d'un souffle. Aniss la plaque, sans parler. Il attend la deuxième tasse. Voilà, c'est posé. Ton dessin peut s'asseoir. Il sèche au soleil du pain. On croque, et lui sèche. Une goutte meurt sur la croûte, minuscule. Sa main sent le tiède du rebord. [pause]</t>
+          <t>Aniss apporte l'ardoise mouillée vers le pain, à la fenêtre. Le rebord est étroit. On mange avec lui ! Papa pose deux tasses, et compte à voix haute. L'ardoise glisse d'un souffle. Aniss la retient, sans parler. Il attend la deuxième tasse. Voilà, c'est posé. Ton dessin peut s'asseoir. Il sèche au soleil du pain. On croque, et lui sèche. Une goutte meurt sur la croûte, minuscule. Sa main sent le tiède du rebord. [pause]</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -13778,7 +13778,7 @@
 enfant-m|On mange avec lui !
 narrateur|Papa pose deux tasses, et compte à voix haute.
 narrateur|L'ardoise glisse d'un souffle.
-narrateur|Aniss la plaque, sans parler.
+narrateur|Aniss la retient, sans parler.
 narrateur|Il attend la deuxième tasse.
 papa|Voilà, c'est posé.
 papa|Ton dessin peut s'asseoir.
@@ -13817,17 +13817,17 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec l'éponge, puis le pain. On a entendu toute ta phrase. Sa main sent le rebord, et un peu d'eau. Ils croquent près de la fenêtre ; le dessin sèche.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec l'éponge, puis le pain. Tes mots sont arrivés, cette fois. Sa main sent le rebord, et un peu d'eau. Ils croquent près de la fenêtre ; le dessin sèche.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec l'éponge, puis le pain. On a entendu toute ta phrase. Sa main sent le rebord, et un peu d'eau. Ils croquent près de la fenêtre ; le dessin sèche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec l'éponge, puis le pain. Tes mots sont arrivés, cette fois. Sa main sent le rebord, et un peu d'eau. Ils croquent près de la fenêtre ; le dessin sèche.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec l'éponge, puis le pain. On a entendu toute ta phrase. Sa main sent le rebord, et un peu d'eau. Ils croquent près de la fenêtre ; le dessin sèche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec l'éponge, puis le pain. Tes mots sont arrivés, cette fois. Sa main sent le rebord, et un peu d'eau. Ils croquent près de la fenêtre ; le dessin sèche.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -13965,7 +13965,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné près de la fenêtre, avec l'éponge, puis le pain.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Sa main sent le rebord, et un peu d'eau.
 narrateur|Ils croquent près de la fenêtre ; le dessin sèche.</t>
         </is>
@@ -14187,17 +14187,17 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec l'éponge, puis le volet. On a entendu toute ta phrase. Sa main sent le rebord, et un peu d'eau. L'éponge et le volet sentent l'eau et le bois.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec l'éponge, puis le volet. Tes mots sont arrivés, cette fois. Sa main sent le rebord, et un peu d'eau. L'éponge et le volet sentent l'eau et le bois.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec l'éponge, puis le volet. On a entendu toute ta phrase. Sa main sent le rebord, et un peu d'eau. L'éponge et le volet sentent l'eau et le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec l'éponge, puis le volet. Tes mots sont arrivés, cette fois. Sa main sent le rebord, et un peu d'eau. L'éponge et le volet sentent l'eau et le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec l'éponge, puis le volet. On a entendu toute ta phrase. Sa main sent le rebord, et un peu d'eau. L'éponge et le volet sentent l'eau et le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec l'éponge, puis le volet. Tes mots sont arrivés, cette fois. Sa main sent le rebord, et un peu d'eau. L'éponge et le volet sentent l'eau et le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr"/>
@@ -14335,7 +14335,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné près de la fenêtre, avec l'éponge, puis le volet.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Sa main sent le rebord, et un peu d'eau.
 narrateur|L'éponge et le volet sentent l'eau et le bois.</t>
         </is>
@@ -14759,17 +14759,17 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>La craie jaune veut un dernier point, sous le clou. Aniss parle pendant que maman ouvre. Un soleil, juste là ! Le volet prend sa phrase. Le soleil devient une virgule. Aniss attend que le bois s'arrête. Recommence le soleil. Un rond jaune s'installe, propre. Il chauffe le cerf-volant du mur. Une virgule jaune reste sous le clou, en trop. Aniss la chasse d'un doigt. Sa main porte un petit astre. Le clou a son étoile.</t>
+          <t>La craie jaune veut un dernier point, sous le clou. Aniss parle pendant que maman ouvre. Un soleil, juste là ! Le volet prend sa phrase. Le soleil devient une virgule. Aniss attend que le bois s'arrête. Recommence le soleil. Un rond jaune s'installe, propre. Il chauffe le cerf-volant du mur. Une virgule jaune reste sous le clou, en trop. Aniss la chasse d'un doigt. Sa main porte un petit soleil. Le clou a son étoile.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La craie jaune veut un dernier point, sous le clou. Aniss parle pendant que maman ouvre. Un soleil, juste là ! Le volet prend sa phrase. Le soleil devient une virgule. Aniss attend que le bois s'arrête. Recommence le soleil. Un rond jaune s'installe, propre. Il chauffe le cerf-volant du mur. Une virgule jaune reste sous le clou, en trop. Aniss la chasse d'un doigt. Sa main porte un petit astre. Le clou a son étoile.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La craie jaune veut un dernier point, sous le clou. Aniss parle pendant que maman ouvre. Un soleil, juste là ! Le volet prend sa phrase. Le soleil devient une virgule. Aniss attend que le bois s'arrête. Recommence le soleil. Un rond jaune s'installe, propre. Il chauffe le cerf-volant du mur. Une virgule jaune reste sous le clou, en trop. Aniss la chasse d'un doigt. Sa main porte un petit soleil. Le clou a son étoile.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>La craie jaune veut un dernier point, sous le clou. Aniss parle pendant que maman ouvre. Un soleil, juste là ! Le volet prend sa phrase. Le soleil devient une virgule. Aniss attend que le bois s'arrête. Recommence le soleil. Un rond jaune s'installe, propre. Il chauffe le cerf-volant du mur. Une virgule jaune reste sous le clou, en trop. Aniss la chasse d'un doigt. Sa main porte un petit astre. Le clou a son étoile. [pause]</t>
+          <t>La craie jaune veut un dernier point, sous le clou. Aniss parle pendant que maman ouvre. Un soleil, juste là ! Le volet prend sa phrase. Le soleil devient une virgule. Aniss attend que le bois s'arrête. Recommence le soleil. Un rond jaune s'installe, propre. Il chauffe le cerf-volant du mur. Une virgule jaune reste sous le clou, en trop. Aniss la chasse d'un doigt. Sa main porte un petit soleil. Le clou a son étoile. [pause]</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
@@ -14914,7 +14914,7 @@
 enfant-m|Il chauffe le cerf-volant du mur.
 papa|Une virgule jaune reste sous le clou, en trop.
 narrateur|Aniss la chasse d'un doigt.
-narrateur|Sa main porte un petit astre.
+narrateur|Sa main porte un petit soleil.
 maman|Le clou a son étoile.</t>
         </is>
       </c>
@@ -14947,17 +14947,17 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec la craie neuve, puis le clou. On a entendu toute ta phrase. Un grain de craie lui tient lieu d'anneau. Une virgule jaune de craie reste sous le clou.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec la craie neuve, puis le clou. Tes mots sont arrivés, cette fois. Un grain de craie lui tient lieu d'anneau. Une virgule jaune de craie reste sous le clou.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec la craie neuve, puis le clou. On a entendu toute ta phrase. Un grain de craie lui tient lieu d'anneau. Une virgule jaune de craie reste sous le clou.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec la craie neuve, puis le clou. Tes mots sont arrivés, cette fois. Un grain de craie lui tient lieu d'anneau. Une virgule jaune de craie reste sous le clou.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec la craie neuve, puis le clou. On a entendu toute ta phrase. Un grain de craie lui tient lieu d'anneau. Une virgule jaune de craie reste sous le clou.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec la craie neuve, puis le clou. Tes mots sont arrivés, cette fois. Un grain de craie lui tient lieu d'anneau. Une virgule jaune de craie reste sous le clou.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
@@ -15095,7 +15095,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné près de la fenêtre, avec la craie neuve, puis le clou.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Un grain de craie lui tient lieu d'anneau.
 narrateur|Une virgule jaune de craie reste sous le clou.</t>
         </is>
@@ -15317,17 +15317,17 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec la craie neuve, puis le pain. On a entendu toute ta phrase. Un grain de craie lui tient lieu d'anneau. Derrière le pain, le vrai cerf-volant rouge salue la vitre.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec la craie neuve, puis le pain. Tes mots sont arrivés, cette fois. Un grain de craie lui tient lieu d'anneau. Derrière le pain, le vrai cerf-volant rouge salue la vitre.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec la craie neuve, puis le pain. On a entendu toute ta phrase. Un grain de craie lui tient lieu d'anneau. Derrière le pain, le vrai cerf-volant rouge salue la vitre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec la craie neuve, puis le pain. Tes mots sont arrivés, cette fois. Un grain de craie lui tient lieu d'anneau. Derrière le pain, le vrai cerf-volant rouge salue la vitre.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec la craie neuve, puis le pain. On a entendu toute ta phrase. Un grain de craie lui tient lieu d'anneau. Derrière le pain, le vrai cerf-volant rouge salue la vitre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec la craie neuve, puis le pain. Tes mots sont arrivés, cette fois. Un grain de craie lui tient lieu d'anneau. Derrière le pain, le vrai cerf-volant rouge salue la vitre.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr"/>
@@ -15465,7 +15465,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné près de la fenêtre, avec la craie neuve, puis le pain.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Un grain de craie lui tient lieu d'anneau.
 narrateur|Derrière le pain, le vrai cerf-volant rouge salue la vitre.</t>
         </is>
@@ -15687,17 +15687,17 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec la craie neuve, puis le volet. On a entendu toute ta phrase. Un grain de craie lui tient lieu d'anneau. Deux cerfs-volants se regardent : l'un rouge, l'un blanc.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec la craie neuve, puis le volet. Tes mots sont arrivés, cette fois. Un grain de craie lui tient lieu d'anneau. Deux cerfs-volants se regardent : l'un rouge, l'un blanc.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec la craie neuve, puis le volet. On a entendu toute ta phrase. Un grain de craie lui tient lieu d'anneau. Deux cerfs-volants se regardent : l'un rouge, l'un blanc.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec la craie neuve, puis le volet. Tes mots sont arrivés, cette fois. Un grain de craie lui tient lieu d'anneau. Deux cerfs-volants se regardent : l'un rouge, l'un blanc.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec la craie neuve, puis le volet. On a entendu toute ta phrase. Un grain de craie lui tient lieu d'anneau. Deux cerfs-volants se regardent : l'un rouge, l'un blanc.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec la craie neuve, puis le volet. Tes mots sont arrivés, cette fois. Un grain de craie lui tient lieu d'anneau. Deux cerfs-volants se regardent : l'un rouge, l'un blanc.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr"/>
@@ -15835,7 +15835,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné près de la fenêtre, avec la craie neuve, puis le volet.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Un grain de craie lui tient lieu d'anneau.
 narrateur|Deux cerfs-volants se regardent : l'un rouge, l'un blanc.</t>
         </is>
@@ -16447,17 +16447,17 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec le tabouret, puis le clou. On a entendu toute ta phrase. Sa main quitte le loquet, sans se presser. Aniss accroche l'ardoise sans redescendre du tabouret.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec le tabouret, puis le clou. Tes mots sont arrivés, cette fois. Sa main quitte le loquet, sans se presser. Aniss accroche l'ardoise sans redescendre du tabouret.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec le tabouret, puis le clou. On a entendu toute ta phrase. Sa main quitte le loquet, sans se presser. Aniss accroche l'ardoise sans redescendre du tabouret.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec le tabouret, puis le clou. Tes mots sont arrivés, cette fois. Sa main quitte le loquet, sans se presser. Aniss accroche l'ardoise sans redescendre du tabouret.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec le tabouret, puis le clou. On a entendu toute ta phrase. Sa main quitte le loquet, sans se presser. Aniss accroche l'ardoise sans redescendre du tabouret.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec le tabouret, puis le clou. Tes mots sont arrivés, cette fois. Sa main quitte le loquet, sans se presser. Aniss accroche l'ardoise sans redescendre du tabouret.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -16595,7 +16595,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné près de la fenêtre, avec le tabouret, puis le clou.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Sa main quitte le loquet, sans se presser.
 narrateur|Aniss accroche l'ardoise sans redescendre du tabouret.</t>
         </is>
@@ -16817,17 +16817,17 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec le tabouret, puis le pain. On a entendu toute ta phrase. Sa main quitte le loquet, sans se presser. Le pain reste sur le rebord, l'ardoise sur ses genoux.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec le tabouret, puis le pain. Tes mots sont arrivés, cette fois. Sa main quitte le loquet, sans se presser. Le pain reste sur le rebord, l'ardoise sur ses genoux.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec le tabouret, puis le pain. On a entendu toute ta phrase. Sa main quitte le loquet, sans se presser. Le pain reste sur le rebord, l'ardoise sur ses genoux.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec le tabouret, puis le pain. Tes mots sont arrivés, cette fois. Sa main quitte le loquet, sans se presser. Le pain reste sur le rebord, l'ardoise sur ses genoux.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec le tabouret, puis le pain. On a entendu toute ta phrase. Sa main quitte le loquet, sans se presser. Le pain reste sur le rebord, l'ardoise sur ses genoux.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec le tabouret, puis le pain. Tes mots sont arrivés, cette fois. Sa main quitte le loquet, sans se presser. Le pain reste sur le rebord, l'ardoise sur ses genoux.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr"/>
@@ -16965,7 +16965,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné près de la fenêtre, avec le tabouret, puis le pain.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Sa main quitte le loquet, sans se presser.
 narrateur|Le pain reste sur le rebord, l'ardoise sur ses genoux.</t>
         </is>
@@ -16999,17 +16999,17 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Aniss, tabouret et volet, veut tenir trois choses. L'ardoise, le loquet, et sa phrase. Regardez les trois ! Le vent, papa, et lui parlent ensemble. Rien n'est clair. Aniss choisit le silence, une seconde. On se tait. Montre. Le tabouret, le volet, et ma main. Trois choses sages, et un cerf-volant. Le bois, le bois, et la peau se tiennent. Dehors, le rouge reste, pour un peu. Sa main, au loquet, ne serre plus trop.</t>
+          <t>Aniss, tabouret et volet, veut tenir trois choses. L'ardoise, le loquet, et sa phrase. Regardez les trois ! Le vent, papa, et lui parlent ensemble. Rien n'est clair. Aniss choisit le silence, une seconde. On se tait. Montre. Le tabouret, le volet, et ma main. Trois choses sages, et un cerf-volant. Tabouret, volet, et main restent collés. Dehors, le rouge reste, pour un peu. Sa main, au loquet, ne serre plus trop.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss, tabouret et volet, veut tenir trois choses. L'ardoise, le loquet, et sa phrase. Regardez les trois ! Le vent, papa, et lui parlent ensemble. Rien n'est clair. Aniss choisit le silence, une seconde. On se tait. Montre. Le tabouret, le volet, et ma main. Trois choses sages, et un cerf-volant. Le bois, le bois, et la peau se tiennent. Dehors, le rouge reste, pour un peu. Sa main, au loquet, ne serre plus trop.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss, tabouret et volet, veut tenir trois choses. L'ardoise, le loquet, et sa phrase. Regardez les trois ! Le vent, papa, et lui parlent ensemble. Rien n'est clair. Aniss choisit le silence, une seconde. On se tait. Montre. Le tabouret, le volet, et ma main. Trois choses sages, et un cerf-volant. Tabouret, volet, et main restent collés. Dehors, le rouge reste, pour un peu. Sa main, au loquet, ne serre plus trop.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Aniss, tabouret et volet, veut tenir trois choses. L'ardoise, le loquet, et sa phrase. Regardez les trois ! Le vent, papa, et lui parlent ensemble. Rien n'est clair. Aniss choisit le silence, une seconde. On se tait. Montre. Le tabouret, le volet, et ma main. Trois choses sages, et un cerf-volant. Le bois, le bois, et la peau se tiennent. Dehors, le rouge reste, pour un peu. Sa main, au loquet, ne serre plus trop. [pause]</t>
+          <t>Aniss, tabouret et volet, veut tenir trois choses. L'ardoise, le loquet, et sa phrase. Regardez les trois ! Le vent, papa, et lui parlent ensemble. Rien n'est clair. Aniss choisit le silence, une seconde. On se tait. Montre. Le tabouret, le volet, et ma main. Trois choses sages, et un cerf-volant. Tabouret, volet, et main restent collés. Dehors, le rouge reste, pour un peu. Sa main, au loquet, ne serre plus trop. [pause]</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -17153,7 +17153,7 @@
 papa|Montre.
 enfant-m|Le tabouret, le volet, et ma main.
 maman|Trois choses sages, et un cerf-volant.
-narrateur|Le bois, le bois, et la peau se tiennent.
+narrateur|Tabouret, volet, et main restent collés.
 narrateur|Dehors, le rouge reste, pour un peu.
 narrateur|Sa main, au loquet, ne serre plus trop.</t>
         </is>
@@ -17187,17 +17187,17 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec le tabouret, puis le volet. On a entendu toute ta phrase. Sa main quitte le loquet, sans se presser. Le tabouret, le volet, et sa main restent tranquilles.</t>
+          <t>Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec le tabouret, puis le volet. Tes mots sont arrivés, cette fois. Sa main quitte le loquet, sans se presser. Le tabouret, le volet, et sa main restent tranquilles.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec le tabouret, puis le volet. On a entendu toute ta phrase. Sa main quitte le loquet, sans se presser. Le tabouret, le volet, et sa main restent tranquilles.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec le tabouret, puis le volet. Tes mots sont arrivés, cette fois. Sa main quitte le loquet, sans se presser. Le tabouret, le volet, et sa main restent tranquilles.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec le tabouret, puis le volet. On a entendu toute ta phrase. Sa main quitte le loquet, sans se presser. Le tabouret, le volet, et sa main restent tranquilles.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Plus tard, le pain est sur la table, et le soleil baisse. À toi, Aniss. Nous t'écoutons jusqu'au bout. J'ai dessiné près de la fenêtre, avec le tabouret, puis le volet. Tes mots sont arrivés, cette fois. Sa main quitte le loquet, sans se presser. Le tabouret, le volet, et sa main restent tranquilles.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr"/>
@@ -17335,7 +17335,7 @@
 papa|À toi, Aniss.
 papa|Nous t'écoutons jusqu'au bout.
 enfant-m|J'ai dessiné près de la fenêtre, avec le tabouret, puis le volet.
-maman|On a entendu toute ta phrase.
+maman|Tes mots sont arrivés, cette fois.
 narrateur|Sa main quitte le loquet, sans se presser.
 narrateur|Le tabouret, le volet, et sa main restent tranquilles.</t>
         </is>
@@ -17363,7 +17363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17476,6 +17476,13 @@
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>